<commit_message>
updated BOM and robot model
</commit_message>
<xml_diff>
--- a/docs/bom.xlsx
+++ b/docs/bom.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
   <si>
     <t xml:space="preserve">BOM</t>
   </si>
@@ -52,7 +52,7 @@
     <t xml:space="preserve">Sensore di distanza a luce IR </t>
   </si>
   <si>
-    <t xml:space="preserve">BNo085 imu</t>
+    <t xml:space="preserve">IMU MPU6050</t>
   </si>
   <si>
     <t xml:space="preserve">Sensore di orientamento axis XYZ</t>
@@ -80,6 +80,12 @@
   </si>
   <si>
     <t xml:space="preserve">MPU per elaborazione immagini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GM25 Gear Motor Mounting Bracket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bracket per motori</t>
   </si>
   <si>
     <t xml:space="preserve">TOTALE</t>
@@ -310,7 +316,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -384,6 +390,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -677,7 +703,7 @@
   <dimension ref="B2:K1048576"/>
   <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="55.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="55.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.96"/>
@@ -748,14 +774,14 @@
         <v>4.89</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">PRODUCT(C$5,D$5)</f>
-        <v>14.67</v>
+        <v>24.45</v>
       </c>
       <c r="G5" s="7" t="n">
         <f aca="false">PRODUCT(C$5,E$5)</f>
@@ -776,21 +802,21 @@
         <v>10</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>12.49</v>
+        <v>2.11</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" s="12" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="11" t="n">
         <f aca="false">PRODUCT(C$6,D$6)</f>
-        <v>12.49</v>
+        <v>4.22</v>
       </c>
       <c r="G6" s="11" t="n">
         <f aca="false">PRODUCT(C$6,E$6)</f>
-        <v>12.49</v>
+        <v>2.11</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>11</v>
@@ -798,7 +824,7 @@
       <c r="I6" s="12"/>
       <c r="J6" s="12"/>
       <c r="K6" s="13" t="str">
-        <f aca="false">HYPERLINK("https://it.aliexpress.com/item/1005008036466921.html", "AliExpress")</f>
+        <f aca="false">HYPERLINK("https://it.aliexpress.com/item/1005010057794277.html", "AliExpress")</f>
         <v>AliExpress</v>
       </c>
     </row>
@@ -841,14 +867,14 @@
         <v>17.52</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="n">
         <f aca="false">PRODUCT(C$8,D$8)</f>
-        <v>35.04</v>
+        <v>70.08</v>
       </c>
       <c r="G8" s="11" t="n">
         <f aca="false">PRODUCT(C$8,E$8)</f>
@@ -926,150 +952,200 @@
         <v>Ebay</v>
       </c>
     </row>
+    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <f aca="false">D8</f>
+        <v>4</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="20" t="n">
+        <f aca="false">PRODUCT(C$11:D$11)</f>
+        <v>12</v>
+      </c>
+      <c r="G11" s="20" t="n">
+        <f aca="false">PRODUCT(C$11,E$11)</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="22"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="23" t="str">
+        <f aca="false">HYPERLINK("https://microdcmotors.com/product/gm25-gear-motor-mounting-bracket-stand","ChineHobbyLine")</f>
+        <v>ChineHobbyLine</v>
+      </c>
+    </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="2"/>
-      <c r="E12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
+      <c r="B12" s="0"/>
+      <c r="C12" s="0"/>
+      <c r="D12" s="0"/>
+      <c r="E12" s="0"/>
+      <c r="F12" s="0"/>
+      <c r="G12" s="0"/>
+      <c r="K12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
+      <c r="B13" s="0"/>
+      <c r="C13" s="0"/>
+      <c r="D13" s="0"/>
+      <c r="E13" s="0"/>
+      <c r="F13" s="0"/>
+      <c r="G13" s="0"/>
+      <c r="K13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="20" t="n">
-        <f aca="false">SUM(D$5:D$10)</f>
-        <v>13</v>
-      </c>
-      <c r="E14" s="3" t="s">
+      <c r="C14" s="2"/>
+      <c r="E14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="4" t="s">
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="C16" s="25" t="n">
+        <f aca="false">SUM(D$5:D$11)</f>
+        <v>22</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="F16" s="3"/>
+      <c r="G16" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="J14" s="5"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="21" t="s">
+      <c r="H16" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="9" t="n">
-        <f aca="false">SUM(E$5:E$10)</f>
+      <c r="I16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <f aca="false">SUM(E$5:E$11)</f>
         <v>4</v>
       </c>
-      <c r="E15" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="F15" s="22"/>
-      <c r="G15" s="23" t="n">
+      <c r="E17" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="27"/>
+      <c r="G17" s="28" t="n">
         <v>150</v>
       </c>
-      <c r="H15" s="24" t="n">
-        <f aca="false">IF(C17&gt;G15,TRUE())</f>
+      <c r="H17" s="29" t="n">
+        <f aca="false">IF(C19&gt;G17,TRUE())</f>
         <v>1</v>
       </c>
-      <c r="I15" s="25" t="n">
-        <f aca="false">IF(C19&gt;G15,TRUE())</f>
+      <c r="I17" s="30" t="n">
+        <f aca="false">IF(C21&gt;G17,TRUE())</f>
         <v>1</v>
       </c>
-      <c r="J15" s="25"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="14" t="n">
-        <f aca="false">SUM(C14:C15)</f>
-        <v>17</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="F16" s="15"/>
-      <c r="G16" s="27" t="n">
+      <c r="J17" s="30"/>
+    </row>
+    <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <f aca="false">SUM(C16:C17)</f>
+        <v>26</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" s="15"/>
+      <c r="G18" s="32" t="n">
         <v>200</v>
       </c>
-      <c r="H16" s="28" t="n">
-        <f aca="false">IF(C17&gt;G16,TRUE())</f>
-        <v>0</v>
-      </c>
-      <c r="I16" s="29" t="n">
-        <f aca="false">IF(C19&gt;G16,TRUE())</f>
+      <c r="H18" s="33" t="n">
+        <f aca="false">IF(C19&gt;G18,TRUE())</f>
         <v>1</v>
       </c>
-      <c r="J16" s="29"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="31" t="n">
-        <f aca="false">SUM(F$5:F$10)</f>
-        <v>196.89</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="32" t="n">
+      <c r="I18" s="34" t="n">
+        <f aca="false">IF(C21&gt;G18,TRUE())</f>
+        <v>1</v>
+      </c>
+      <c r="J18" s="34"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="36" t="n">
+        <f aca="false">SUM(F$5:F$11)</f>
+        <v>245.44</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="37" t="n">
         <f aca="false">SUM(G5:G10)</f>
-        <v>36.62</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="C19" s="33" t="n">
-        <f aca="false">SUM(C17:C18)</f>
-        <v>233.51</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C20" s="34" t="n">
-        <f aca="false">QUOTIENT(C$17,3)</f>
-        <v>65</v>
+        <v>26.24</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="36" t="n">
+      <c r="C21" s="38" t="n">
+        <f aca="false">SUM(C19:C20)</f>
+        <v>271.68</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="39" t="n">
         <f aca="false">QUOTIENT(C$19,3)</f>
-        <v>77</v>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="41" t="n">
+        <f aca="false">QUOTIENT(C$21,3)</f>
+        <v>90</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E25" s="37"/>
+      <c r="E25" s="42"/>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H26" s="1"/>
@@ -1078,7 +1154,7 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="B2:K3"/>
     <mergeCell ref="H4:J4"/>
     <mergeCell ref="H5:J5"/>
@@ -1087,21 +1163,22 @@
     <mergeCell ref="H8:J8"/>
     <mergeCell ref="H9:J9"/>
     <mergeCell ref="H10:J10"/>
-    <mergeCell ref="B12:C13"/>
-    <mergeCell ref="E12:J13"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="B14:C15"/>
+    <mergeCell ref="E14:J15"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="I16:J16"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="I18:J18"/>
   </mergeCells>
-  <conditionalFormatting sqref="H15:I16">
+  <conditionalFormatting sqref="H17:I18">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H15:I16">
+  <conditionalFormatting sqref="H17:I18">
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>1</formula>
     </cfRule>

</xml_diff>